<commit_message>
feat: implement v3 linear rooms and permanent progression
</commit_message>
<xml_diff>
--- a/config/excel/CfgBosses.xlsx
+++ b/config/excel/CfgBosses.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgBosses" sheetId="1" r:id="R1eb83b04fbda4a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgBosses" sheetId="1" r:id="R9239d52f47f84293"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,28 +13,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
-      <x:sz val="10"/>
-      <x:name val="Microsoft YaHei"/>
-    </x:font>
-    <x:font>
       <x:b/>
-      <x:sz val="10"/>
+      <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Microsoft YaHei"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF0000FF"/>
-      <x:name val="Microsoft YaHei"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -46,34 +37,23 @@
         <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFDBEAF7"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF2CC"/>
-      </x:patternFill>
-    </x:fill>
   </x:fills>
   <x:borders count="1">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -275,227 +255,104 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
-  </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" s="2" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" s="2" t="str">
         <x:v>EnemyID</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
-        <x:v>MapID</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="str">
-        <x:v>PoolID</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="str">
-        <x:v>Weight</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
-        <x:v>MinLevel</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="str">
-        <x:v>MaxLevel</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="str">
+      <x:c r="D1" s="2" t="str">
         <x:v>RewardID</x:v>
       </x:c>
-      <x:c r="J1" s="3" t="str">
+      <x:c r="E1" s="2" t="str">
         <x:v>WeaknessDescription</x:v>
       </x:c>
-      <x:c r="K1" s="3" t="str">
+      <x:c r="F1" s="2" t="str">
         <x:v>CollectionPreviewIDs</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="4" t="str">
+    <x:row r="2">
+      <x:c r="A2" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="B2" s="4" t="str">
+      <x:c r="B2" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="C2" s="4" t="str">
+      <x:c r="C2" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="D2" s="4" t="str">
+      <x:c r="D2" t="str">
         <x:v>int</x:v>
       </x:c>
-      <x:c r="E2" s="4" t="str">
+      <x:c r="E2" t="str">
         <x:v>string</x:v>
       </x:c>
-      <x:c r="F2" s="4" t="str">
-        <x:v>int</x:v>
-      </x:c>
-      <x:c r="G2" s="4" t="str">
-        <x:v>int</x:v>
-      </x:c>
-      <x:c r="H2" s="4" t="str">
-        <x:v>int</x:v>
-      </x:c>
-      <x:c r="I2" s="4" t="str">
-        <x:v>int</x:v>
-      </x:c>
-      <x:c r="J2" s="4" t="str">
-        <x:v>string</x:v>
-      </x:c>
-      <x:c r="K2" s="4" t="str">
+      <x:c r="F2" t="str">
         <x:v>string[]</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="42" customHeight="1">
-      <x:c r="A3" s="6" t="str">
-        <x:v># Boss定义编号</x:v>
-      </x:c>
-      <x:c r="B3" s="6" t="str">
-        <x:v>Boss预告名</x:v>
-      </x:c>
-      <x:c r="C3" s="6" t="str">
-        <x:v>战斗敌人定义</x:v>
-      </x:c>
-      <x:c r="D3" s="6" t="str">
-        <x:v>绑定地图资源</x:v>
-      </x:c>
-      <x:c r="E3" s="6" t="str">
-        <x:v>Boss候选池</x:v>
-      </x:c>
-      <x:c r="F3" s="6" t="str">
-        <x:v>抽取权重</x:v>
-      </x:c>
-      <x:c r="G3" s="6" t="str">
-        <x:v>最低关卡等级</x:v>
-      </x:c>
-      <x:c r="H3" s="6" t="str">
-        <x:v>最高关卡等级</x:v>
-      </x:c>
-      <x:c r="I3" s="6" t="str">
-        <x:v>战利品规则</x:v>
-      </x:c>
-      <x:c r="J3" s="6" t="str">
-        <x:v>机制与弱点预告</x:v>
-      </x:c>
-      <x:c r="K3" s="6" t="str">
-        <x:v>专属收藏预览</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="7" t="n">
+    <x:row r="3">
+      <x:c r="A3" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B4" s="7" t="str">
+      <x:c r="B3" t="str">
         <x:v>遗迹守门者</x:v>
       </x:c>
-      <x:c r="C4" s="7" t="n">
+      <x:c r="C3" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D4" s="7" t="n">
+      <x:c r="D3" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E4" s="7" t="str">
-        <x:v>region</x:v>
-      </x:c>
-      <x:c r="F4" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G4" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H4" s="7" t="n">
-        <x:v>1000</x:v>
-      </x:c>
-      <x:c r="I4" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J4" s="7" t="str">
+      <x:c r="E3" t="str">
         <x:v>环形重击前离开范围；流血额外有效。</x:v>
       </x:c>
-      <x:c r="K4" s="7" t="str">
+      <x:c r="F3" t="str">
         <x:v>gate_sigil</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="7" t="n">
+    <x:row r="4">
+      <x:c r="A4" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B5" s="7" t="str">
+      <x:c r="B4" t="str">
         <x:v>庭院双刃统领</x:v>
       </x:c>
-      <x:c r="C5" s="7" t="n">
+      <x:c r="C4" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D5" s="7" t="n">
+      <x:c r="D4" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E5" s="7" t="str">
-        <x:v>region</x:v>
-      </x:c>
-      <x:c r="F5" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G5" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H5" s="7" t="n">
-        <x:v>1000</x:v>
-      </x:c>
-      <x:c r="I5" s="7" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J5" s="7" t="str">
+      <x:c r="E4" t="str">
         <x:v>中距离追击与近身爆发；暴击追伤额外有效。</x:v>
       </x:c>
-      <x:c r="K5" s="7" t="str">
+      <x:c r="F4" t="str">
         <x:v>court_medal</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="7" t="n">
+    <x:row r="5">
+      <x:c r="A5" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="str">
+      <x:c r="B5" t="str">
         <x:v>遗迹核心守望者</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="n">
+      <x:c r="C5" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="D6" s="7" t="n">
+      <x:c r="D5" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E6" s="7" t="str">
-        <x:v>final</x:v>
-      </x:c>
-      <x:c r="F6" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G6" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H6" s="7" t="n">
-        <x:v>1000</x:v>
-      </x:c>
-      <x:c r="I6" s="7" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J6" s="7" t="str">
+      <x:c r="E5" t="str">
         <x:v>后半程冲锋；流血、暴击追伤、反击均有优势。</x:v>
       </x:c>
-      <x:c r="K6" s="7" t="str">
+      <x:c r="F5" t="str">
         <x:v>core_fragment</x:v>
       </x:c>
     </x:row>

</xml_diff>